<commit_message>
[feat/ASP-2677-Add-Percent-to-Module-Swap-Report] Join leyend with formula
</commit_message>
<xml_diff>
--- a/api/templates/module_swaps/en.xlsx
+++ b/api/templates/module_swaps/en.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24931"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B213D06-2BD5-40EA-A592-431EDF03AD0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACB194E-60CC-4FC8-910D-5F85A03AE147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>&lt;Table&gt;</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>Instrument serial</t>
-  </si>
-  <si>
-    <t>Percent Module Swaps within SLA:</t>
   </si>
 </sst>
 </file>
@@ -214,7 +211,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -250,6 +247,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,13 +681,11 @@
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="16" t="s">
-        <v>21</v>
+      <c r="A5" s="16" t="str">
+        <f>+"Percent Module Swaps within SLA: "&amp;TEXT(COUNTIF(D8:D10000,"&lt;=8")/COUNTIF(D8:D10000,"&lt;&gt;"),"0%")</f>
+        <v>Percent Module Swaps within SLA: 0%</v>
       </c>
-      <c r="B5" s="15">
-        <f>COUNTIF(D8:D10000,"&lt;=8")/COUNTIF(D8:D10000,"&lt;&gt;")</f>
-        <v>0</v>
-      </c>
+      <c r="B5" s="15"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
       <c r="E5" s="4"/>
@@ -776,2582 +772,3224 @@
       <c r="G11"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D12" s="17"/>
       <c r="E12"/>
       <c r="G12"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D13" s="17"/>
       <c r="E13"/>
       <c r="G13"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D14" s="17"/>
       <c r="E14"/>
       <c r="G14"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D15" s="17"/>
       <c r="E15"/>
       <c r="G15"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D16" s="17"/>
       <c r="E16"/>
       <c r="G16"/>
     </row>
-    <row r="17" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D17" s="17"/>
       <c r="E17"/>
       <c r="G17"/>
     </row>
-    <row r="18" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D18" s="17"/>
       <c r="E18"/>
       <c r="G18"/>
     </row>
-    <row r="19" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D19" s="17"/>
       <c r="E19"/>
       <c r="G19"/>
     </row>
-    <row r="20" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D20" s="17"/>
       <c r="E20"/>
       <c r="G20"/>
     </row>
-    <row r="21" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="21" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D21" s="17"/>
       <c r="E21"/>
       <c r="G21"/>
     </row>
-    <row r="22" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="22" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D22" s="17"/>
       <c r="E22"/>
       <c r="G22"/>
     </row>
-    <row r="23" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="23" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D23" s="17"/>
       <c r="E23"/>
       <c r="G23"/>
     </row>
-    <row r="24" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="24" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D24" s="17"/>
       <c r="E24"/>
       <c r="G24"/>
     </row>
-    <row r="25" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D25" s="17"/>
       <c r="E25"/>
       <c r="G25"/>
     </row>
-    <row r="26" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D26" s="17"/>
       <c r="E26"/>
       <c r="G26"/>
     </row>
-    <row r="27" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D27" s="17"/>
       <c r="E27"/>
       <c r="G27"/>
     </row>
-    <row r="28" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D28" s="17"/>
       <c r="E28"/>
       <c r="G28"/>
     </row>
-    <row r="29" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D29" s="17"/>
       <c r="E29"/>
       <c r="G29"/>
     </row>
-    <row r="30" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D30" s="17"/>
       <c r="E30"/>
       <c r="G30"/>
     </row>
-    <row r="31" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D31" s="17"/>
       <c r="E31"/>
       <c r="G31"/>
     </row>
-    <row r="32" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D32" s="17"/>
       <c r="E32"/>
       <c r="G32"/>
     </row>
-    <row r="33" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="33" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D33" s="17"/>
       <c r="E33"/>
       <c r="G33"/>
     </row>
-    <row r="34" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="34" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D34" s="17"/>
       <c r="E34"/>
       <c r="G34"/>
     </row>
-    <row r="35" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D35" s="17"/>
       <c r="E35"/>
       <c r="G35"/>
     </row>
-    <row r="36" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="36" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D36" s="17"/>
       <c r="E36"/>
       <c r="G36"/>
     </row>
-    <row r="37" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="37" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D37" s="17"/>
       <c r="E37"/>
       <c r="G37"/>
     </row>
-    <row r="38" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="38" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D38" s="17"/>
       <c r="E38"/>
       <c r="G38"/>
     </row>
-    <row r="39" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="39" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D39" s="17"/>
       <c r="E39"/>
       <c r="G39"/>
     </row>
-    <row r="40" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="40" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D40" s="17"/>
       <c r="E40"/>
       <c r="G40"/>
     </row>
-    <row r="41" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="41" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D41" s="17"/>
       <c r="E41"/>
       <c r="G41"/>
     </row>
-    <row r="42" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="42" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D42" s="17"/>
       <c r="E42"/>
       <c r="G42"/>
     </row>
-    <row r="43" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="43" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D43" s="17"/>
       <c r="E43"/>
       <c r="G43"/>
     </row>
-    <row r="44" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="44" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D44" s="17"/>
       <c r="E44"/>
       <c r="G44"/>
     </row>
-    <row r="45" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="45" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D45" s="17"/>
       <c r="E45"/>
       <c r="G45"/>
     </row>
-    <row r="46" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="46" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D46" s="17"/>
       <c r="E46"/>
       <c r="G46"/>
     </row>
-    <row r="47" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="47" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D47" s="17"/>
       <c r="E47"/>
       <c r="G47"/>
     </row>
-    <row r="48" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="48" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D48" s="17"/>
       <c r="E48"/>
       <c r="G48"/>
     </row>
-    <row r="49" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="49" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D49" s="17"/>
       <c r="E49"/>
       <c r="G49"/>
     </row>
-    <row r="50" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="50" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D50" s="17"/>
       <c r="E50"/>
       <c r="G50"/>
     </row>
-    <row r="51" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="51" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D51" s="17"/>
       <c r="E51"/>
       <c r="G51"/>
     </row>
-    <row r="52" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="52" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D52" s="17"/>
       <c r="E52"/>
       <c r="G52"/>
     </row>
-    <row r="53" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="53" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D53" s="17"/>
       <c r="E53"/>
       <c r="G53"/>
     </row>
-    <row r="54" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="54" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D54" s="17"/>
       <c r="E54"/>
       <c r="G54"/>
     </row>
-    <row r="55" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="55" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D55" s="17"/>
       <c r="E55"/>
       <c r="G55"/>
     </row>
-    <row r="56" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="56" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D56" s="17"/>
       <c r="E56"/>
       <c r="G56"/>
     </row>
-    <row r="57" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="57" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D57" s="17"/>
       <c r="E57"/>
       <c r="G57"/>
     </row>
-    <row r="58" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="58" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D58" s="17"/>
       <c r="E58"/>
       <c r="G58"/>
     </row>
-    <row r="59" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="59" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D59" s="17"/>
       <c r="E59"/>
       <c r="G59"/>
     </row>
-    <row r="60" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="60" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D60" s="17"/>
       <c r="E60"/>
       <c r="G60"/>
     </row>
-    <row r="61" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="61" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D61" s="17"/>
       <c r="E61"/>
       <c r="G61"/>
     </row>
-    <row r="62" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="62" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D62" s="17"/>
       <c r="E62"/>
       <c r="G62"/>
     </row>
-    <row r="63" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="63" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D63" s="17"/>
       <c r="E63"/>
       <c r="G63"/>
     </row>
-    <row r="64" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="64" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D64" s="17"/>
       <c r="E64"/>
       <c r="G64"/>
     </row>
-    <row r="65" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="65" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D65" s="17"/>
       <c r="E65"/>
       <c r="G65"/>
     </row>
-    <row r="66" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="66" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D66" s="17"/>
       <c r="E66"/>
       <c r="G66"/>
     </row>
-    <row r="67" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="67" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D67" s="17"/>
       <c r="E67"/>
       <c r="G67"/>
     </row>
-    <row r="68" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="68" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D68" s="17"/>
       <c r="E68"/>
       <c r="G68"/>
     </row>
-    <row r="69" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="69" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D69" s="17"/>
       <c r="E69"/>
       <c r="G69"/>
     </row>
-    <row r="70" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="70" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D70" s="17"/>
       <c r="E70"/>
       <c r="G70"/>
     </row>
-    <row r="71" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="71" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D71" s="17"/>
       <c r="E71"/>
       <c r="G71"/>
     </row>
-    <row r="72" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="72" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D72" s="17"/>
       <c r="E72"/>
       <c r="G72"/>
     </row>
-    <row r="73" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="73" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D73" s="17"/>
       <c r="E73"/>
       <c r="G73"/>
     </row>
-    <row r="74" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="74" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D74" s="17"/>
       <c r="E74"/>
       <c r="G74"/>
     </row>
-    <row r="75" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="75" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D75" s="17"/>
       <c r="E75"/>
       <c r="G75"/>
     </row>
-    <row r="76" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="76" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D76" s="17"/>
       <c r="E76"/>
       <c r="G76"/>
     </row>
-    <row r="77" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="77" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D77" s="17"/>
       <c r="E77"/>
       <c r="G77"/>
     </row>
-    <row r="78" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="78" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D78" s="17"/>
       <c r="E78"/>
       <c r="G78"/>
     </row>
-    <row r="79" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="79" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D79" s="17"/>
       <c r="E79"/>
       <c r="G79"/>
     </row>
-    <row r="80" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="80" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D80" s="17"/>
       <c r="E80"/>
       <c r="G80"/>
     </row>
-    <row r="81" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="81" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D81" s="17"/>
       <c r="E81"/>
       <c r="G81"/>
     </row>
-    <row r="82" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="82" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D82" s="17"/>
       <c r="E82"/>
       <c r="G82"/>
     </row>
-    <row r="83" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="83" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D83" s="17"/>
       <c r="E83"/>
       <c r="G83"/>
     </row>
-    <row r="84" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="84" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D84" s="17"/>
       <c r="E84"/>
       <c r="G84"/>
     </row>
-    <row r="85" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="85" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D85" s="17"/>
       <c r="E85"/>
       <c r="G85"/>
     </row>
-    <row r="86" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="86" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D86" s="17"/>
       <c r="E86"/>
       <c r="G86"/>
     </row>
-    <row r="87" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="87" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D87" s="17"/>
       <c r="E87"/>
       <c r="G87"/>
     </row>
-    <row r="88" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="88" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D88" s="17"/>
       <c r="E88"/>
       <c r="G88"/>
     </row>
-    <row r="89" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="89" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D89" s="17"/>
       <c r="E89"/>
       <c r="G89"/>
     </row>
-    <row r="90" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="90" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D90" s="17"/>
       <c r="E90"/>
       <c r="G90"/>
     </row>
-    <row r="91" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="91" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D91" s="17"/>
       <c r="E91"/>
       <c r="G91"/>
     </row>
-    <row r="92" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="92" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D92" s="17"/>
       <c r="E92"/>
       <c r="G92"/>
     </row>
-    <row r="93" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="93" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D93" s="17"/>
       <c r="E93"/>
       <c r="G93"/>
     </row>
-    <row r="94" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="94" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D94" s="17"/>
       <c r="E94"/>
       <c r="G94"/>
     </row>
-    <row r="95" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="95" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D95" s="17"/>
       <c r="E95"/>
       <c r="G95"/>
     </row>
-    <row r="96" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="96" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D96" s="17"/>
       <c r="E96"/>
       <c r="G96"/>
     </row>
-    <row r="97" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="97" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D97" s="17"/>
       <c r="E97"/>
       <c r="G97"/>
     </row>
-    <row r="98" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="98" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D98" s="17"/>
       <c r="E98"/>
       <c r="G98"/>
     </row>
-    <row r="99" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="99" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D99" s="17"/>
       <c r="E99"/>
       <c r="G99"/>
     </row>
-    <row r="100" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="100" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D100" s="17"/>
       <c r="E100"/>
       <c r="G100"/>
     </row>
-    <row r="101" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="101" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D101" s="17"/>
       <c r="E101"/>
       <c r="G101"/>
     </row>
-    <row r="102" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="102" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D102" s="17"/>
       <c r="E102"/>
       <c r="G102"/>
     </row>
-    <row r="103" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="103" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D103" s="17"/>
       <c r="E103"/>
       <c r="G103"/>
     </row>
-    <row r="104" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="104" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D104" s="17"/>
       <c r="E104"/>
       <c r="G104"/>
     </row>
-    <row r="105" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="105" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D105" s="17"/>
       <c r="E105"/>
       <c r="G105"/>
     </row>
-    <row r="106" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="106" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D106" s="17"/>
       <c r="E106"/>
       <c r="G106"/>
     </row>
-    <row r="107" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="107" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D107" s="17"/>
       <c r="E107"/>
       <c r="G107"/>
     </row>
-    <row r="108" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="108" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D108" s="17"/>
       <c r="E108"/>
       <c r="G108"/>
     </row>
-    <row r="109" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="109" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D109" s="17"/>
       <c r="E109"/>
       <c r="G109"/>
     </row>
-    <row r="110" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="110" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D110" s="17"/>
       <c r="E110"/>
       <c r="G110"/>
     </row>
-    <row r="111" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="111" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D111" s="17"/>
       <c r="E111"/>
       <c r="G111"/>
     </row>
-    <row r="112" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="112" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D112" s="17"/>
       <c r="E112"/>
       <c r="G112"/>
     </row>
-    <row r="113" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="113" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D113" s="17"/>
       <c r="E113"/>
       <c r="G113"/>
     </row>
-    <row r="114" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="114" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D114" s="17"/>
       <c r="E114"/>
       <c r="G114"/>
     </row>
-    <row r="115" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="115" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D115" s="17"/>
       <c r="E115"/>
       <c r="G115"/>
     </row>
-    <row r="116" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="116" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D116" s="17"/>
       <c r="E116"/>
       <c r="G116"/>
     </row>
-    <row r="117" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="117" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D117" s="17"/>
       <c r="E117"/>
       <c r="G117"/>
     </row>
-    <row r="118" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="118" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D118" s="17"/>
       <c r="E118"/>
       <c r="G118"/>
     </row>
-    <row r="119" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="119" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D119" s="17"/>
       <c r="E119"/>
       <c r="G119"/>
     </row>
-    <row r="120" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="120" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D120" s="17"/>
       <c r="E120"/>
       <c r="G120"/>
     </row>
-    <row r="121" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="121" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D121" s="17"/>
       <c r="E121"/>
       <c r="G121"/>
     </row>
-    <row r="122" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="122" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D122" s="17"/>
       <c r="E122"/>
       <c r="G122"/>
     </row>
-    <row r="123" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="123" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D123" s="17"/>
       <c r="E123"/>
       <c r="G123"/>
     </row>
-    <row r="124" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="124" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D124" s="17"/>
       <c r="E124"/>
       <c r="G124"/>
     </row>
-    <row r="125" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="125" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D125" s="17"/>
       <c r="E125"/>
       <c r="G125"/>
     </row>
-    <row r="126" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="126" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D126" s="17"/>
       <c r="E126"/>
       <c r="G126"/>
     </row>
-    <row r="127" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="127" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D127" s="17"/>
       <c r="E127"/>
       <c r="G127"/>
     </row>
-    <row r="128" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="128" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D128" s="17"/>
       <c r="E128"/>
       <c r="G128"/>
     </row>
-    <row r="129" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="129" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D129" s="17"/>
       <c r="E129"/>
       <c r="G129"/>
     </row>
-    <row r="130" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="130" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D130" s="17"/>
       <c r="E130"/>
       <c r="G130"/>
     </row>
-    <row r="131" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="131" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D131" s="17"/>
       <c r="E131"/>
       <c r="G131"/>
     </row>
-    <row r="132" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="132" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D132" s="17"/>
       <c r="E132"/>
       <c r="G132"/>
     </row>
-    <row r="133" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="133" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D133" s="17"/>
       <c r="E133"/>
       <c r="G133"/>
     </row>
-    <row r="134" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="134" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D134" s="17"/>
       <c r="E134"/>
       <c r="G134"/>
     </row>
-    <row r="135" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="135" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D135" s="17"/>
       <c r="E135"/>
       <c r="G135"/>
     </row>
-    <row r="136" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="136" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D136" s="17"/>
       <c r="E136"/>
       <c r="G136"/>
     </row>
-    <row r="137" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="137" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D137" s="17"/>
       <c r="E137"/>
       <c r="G137"/>
     </row>
-    <row r="138" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="138" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D138" s="17"/>
       <c r="E138"/>
       <c r="G138"/>
     </row>
-    <row r="139" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="139" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D139" s="17"/>
       <c r="E139"/>
       <c r="G139"/>
     </row>
-    <row r="140" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="140" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D140" s="17"/>
       <c r="E140"/>
       <c r="G140"/>
     </row>
-    <row r="141" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="141" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D141" s="17"/>
       <c r="E141"/>
       <c r="G141"/>
     </row>
-    <row r="142" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="142" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D142" s="17"/>
       <c r="E142"/>
       <c r="G142"/>
     </row>
-    <row r="143" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="143" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D143" s="17"/>
       <c r="E143"/>
       <c r="G143"/>
     </row>
-    <row r="144" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="144" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D144" s="17"/>
       <c r="E144"/>
       <c r="G144"/>
     </row>
-    <row r="145" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="145" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D145" s="17"/>
       <c r="E145"/>
       <c r="G145"/>
     </row>
-    <row r="146" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="146" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D146" s="17"/>
       <c r="E146"/>
       <c r="G146"/>
     </row>
-    <row r="147" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="147" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D147" s="17"/>
       <c r="E147"/>
       <c r="G147"/>
     </row>
-    <row r="148" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="148" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D148" s="17"/>
       <c r="E148"/>
       <c r="G148"/>
     </row>
-    <row r="149" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D149" s="17"/>
       <c r="E149"/>
       <c r="G149"/>
     </row>
-    <row r="150" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D150" s="17"/>
       <c r="E150"/>
       <c r="G150"/>
     </row>
-    <row r="151" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D151" s="17"/>
       <c r="E151"/>
       <c r="G151"/>
     </row>
-    <row r="152" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="152" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D152" s="17"/>
       <c r="E152"/>
       <c r="G152"/>
     </row>
-    <row r="153" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="153" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D153" s="17"/>
       <c r="E153"/>
       <c r="G153"/>
     </row>
-    <row r="154" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="154" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D154" s="17"/>
       <c r="E154"/>
       <c r="G154"/>
     </row>
-    <row r="155" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="155" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D155" s="17"/>
       <c r="E155"/>
       <c r="G155"/>
     </row>
-    <row r="156" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="156" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D156" s="17"/>
       <c r="E156"/>
       <c r="G156"/>
     </row>
-    <row r="157" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="157" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D157" s="17"/>
       <c r="E157"/>
       <c r="G157"/>
     </row>
-    <row r="158" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="158" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D158" s="17"/>
       <c r="E158"/>
       <c r="G158"/>
     </row>
-    <row r="159" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="159" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D159" s="17"/>
       <c r="E159"/>
       <c r="G159"/>
     </row>
-    <row r="160" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="160" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D160" s="17"/>
       <c r="E160"/>
       <c r="G160"/>
     </row>
-    <row r="161" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="161" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D161" s="17"/>
       <c r="E161"/>
       <c r="G161"/>
     </row>
-    <row r="162" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="162" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D162" s="17"/>
       <c r="E162"/>
       <c r="G162"/>
     </row>
-    <row r="163" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="163" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D163" s="17"/>
       <c r="E163"/>
       <c r="G163"/>
     </row>
-    <row r="164" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="164" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D164" s="17"/>
       <c r="E164"/>
       <c r="G164"/>
     </row>
-    <row r="165" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="165" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D165" s="17"/>
       <c r="E165"/>
       <c r="G165"/>
     </row>
-    <row r="166" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="166" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D166" s="17"/>
       <c r="E166"/>
       <c r="G166"/>
     </row>
-    <row r="167" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="167" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D167" s="17"/>
       <c r="E167"/>
       <c r="G167"/>
     </row>
-    <row r="168" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="168" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D168" s="17"/>
       <c r="E168"/>
       <c r="G168"/>
     </row>
-    <row r="169" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="169" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D169" s="17"/>
       <c r="E169"/>
       <c r="G169"/>
     </row>
-    <row r="170" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="170" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D170" s="17"/>
       <c r="E170"/>
       <c r="G170"/>
     </row>
-    <row r="171" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="171" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D171" s="17"/>
       <c r="E171"/>
       <c r="G171"/>
     </row>
-    <row r="172" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="172" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D172" s="17"/>
       <c r="E172"/>
       <c r="G172"/>
     </row>
-    <row r="173" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="173" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D173" s="17"/>
       <c r="E173"/>
       <c r="G173"/>
     </row>
-    <row r="174" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="174" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D174" s="17"/>
       <c r="E174"/>
       <c r="G174"/>
     </row>
-    <row r="175" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="175" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D175" s="17"/>
       <c r="E175"/>
       <c r="G175"/>
     </row>
-    <row r="176" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="176" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D176" s="17"/>
       <c r="E176"/>
       <c r="G176"/>
     </row>
-    <row r="177" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="177" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D177" s="17"/>
       <c r="E177"/>
       <c r="G177"/>
     </row>
-    <row r="178" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="178" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D178" s="17"/>
       <c r="E178"/>
       <c r="G178"/>
     </row>
-    <row r="179" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="179" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D179" s="17"/>
       <c r="E179"/>
       <c r="G179"/>
     </row>
-    <row r="180" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="180" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D180" s="17"/>
       <c r="E180"/>
       <c r="G180"/>
     </row>
-    <row r="181" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="181" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D181" s="17"/>
       <c r="E181"/>
       <c r="G181"/>
     </row>
-    <row r="182" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="182" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D182" s="17"/>
       <c r="E182"/>
       <c r="G182"/>
     </row>
-    <row r="183" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="183" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D183" s="17"/>
       <c r="E183"/>
       <c r="G183"/>
     </row>
-    <row r="184" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="184" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D184" s="17"/>
       <c r="E184"/>
       <c r="G184"/>
     </row>
-    <row r="185" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="185" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D185" s="17"/>
       <c r="E185"/>
       <c r="G185"/>
     </row>
-    <row r="186" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="186" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D186" s="17"/>
       <c r="E186"/>
       <c r="G186"/>
     </row>
-    <row r="187" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="187" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D187" s="17"/>
       <c r="E187"/>
       <c r="G187"/>
     </row>
-    <row r="188" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="188" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D188" s="17"/>
       <c r="E188"/>
       <c r="G188"/>
     </row>
-    <row r="189" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="189" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D189" s="17"/>
       <c r="E189"/>
       <c r="G189"/>
     </row>
-    <row r="190" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="190" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D190" s="17"/>
       <c r="E190"/>
       <c r="G190"/>
     </row>
-    <row r="191" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="191" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D191" s="17"/>
       <c r="E191"/>
       <c r="G191"/>
     </row>
-    <row r="192" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="192" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D192" s="17"/>
       <c r="E192"/>
       <c r="G192"/>
     </row>
-    <row r="193" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="193" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D193" s="17"/>
       <c r="E193"/>
       <c r="G193"/>
     </row>
-    <row r="194" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="194" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D194" s="17"/>
       <c r="E194"/>
       <c r="G194"/>
     </row>
-    <row r="195" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="195" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D195" s="17"/>
       <c r="E195"/>
       <c r="G195"/>
     </row>
-    <row r="196" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="196" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D196" s="17"/>
       <c r="E196"/>
       <c r="G196"/>
     </row>
-    <row r="197" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="197" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D197" s="17"/>
       <c r="E197"/>
       <c r="G197"/>
     </row>
-    <row r="198" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="198" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D198" s="17"/>
       <c r="E198"/>
       <c r="G198"/>
     </row>
-    <row r="199" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="199" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D199" s="17"/>
       <c r="E199"/>
       <c r="G199"/>
     </row>
-    <row r="200" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="200" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D200" s="17"/>
       <c r="E200"/>
       <c r="G200"/>
     </row>
-    <row r="201" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="201" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D201" s="17"/>
       <c r="E201"/>
       <c r="G201"/>
     </row>
-    <row r="202" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="202" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D202" s="17"/>
       <c r="E202"/>
       <c r="G202"/>
     </row>
-    <row r="203" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="203" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D203" s="17"/>
       <c r="E203"/>
       <c r="G203"/>
     </row>
-    <row r="204" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="204" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D204" s="17"/>
       <c r="E204"/>
       <c r="G204"/>
     </row>
-    <row r="205" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="205" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D205" s="17"/>
       <c r="E205"/>
       <c r="G205"/>
     </row>
-    <row r="206" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="206" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D206" s="17"/>
       <c r="E206"/>
       <c r="G206"/>
     </row>
-    <row r="207" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="207" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D207" s="17"/>
       <c r="E207"/>
       <c r="G207"/>
     </row>
-    <row r="208" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="208" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D208" s="17"/>
       <c r="E208"/>
       <c r="G208"/>
     </row>
-    <row r="209" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="209" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D209" s="17"/>
       <c r="E209"/>
       <c r="G209"/>
     </row>
-    <row r="210" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="210" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D210" s="17"/>
       <c r="E210"/>
       <c r="G210"/>
     </row>
-    <row r="211" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="211" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D211" s="17"/>
       <c r="E211"/>
       <c r="G211"/>
     </row>
-    <row r="212" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="212" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D212" s="17"/>
       <c r="E212"/>
       <c r="G212"/>
     </row>
-    <row r="213" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="213" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D213" s="17"/>
       <c r="E213"/>
       <c r="G213"/>
     </row>
-    <row r="214" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="214" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D214" s="17"/>
       <c r="E214"/>
       <c r="G214"/>
     </row>
-    <row r="215" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="215" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D215" s="17"/>
       <c r="E215"/>
       <c r="G215"/>
     </row>
-    <row r="216" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="216" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D216" s="17"/>
       <c r="E216"/>
       <c r="G216"/>
     </row>
-    <row r="217" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="217" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D217" s="17"/>
       <c r="E217"/>
       <c r="G217"/>
     </row>
-    <row r="218" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="218" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D218" s="17"/>
       <c r="E218"/>
       <c r="G218"/>
     </row>
-    <row r="219" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="219" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D219" s="17"/>
       <c r="E219"/>
       <c r="G219"/>
     </row>
-    <row r="220" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="220" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D220" s="17"/>
       <c r="E220"/>
       <c r="G220"/>
     </row>
-    <row r="221" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="221" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D221" s="17"/>
       <c r="E221"/>
       <c r="G221"/>
     </row>
-    <row r="222" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="222" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D222" s="17"/>
       <c r="E222"/>
       <c r="G222"/>
     </row>
-    <row r="223" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="223" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D223" s="17"/>
       <c r="E223"/>
       <c r="G223"/>
     </row>
-    <row r="224" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="224" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D224" s="17"/>
       <c r="E224"/>
       <c r="G224"/>
     </row>
-    <row r="225" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="225" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D225" s="17"/>
       <c r="E225"/>
       <c r="G225"/>
     </row>
-    <row r="226" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="226" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D226" s="17"/>
       <c r="E226"/>
       <c r="G226"/>
     </row>
-    <row r="227" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="227" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D227" s="17"/>
       <c r="E227"/>
       <c r="G227"/>
     </row>
-    <row r="228" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="228" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D228" s="17"/>
       <c r="E228"/>
       <c r="G228"/>
     </row>
-    <row r="229" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="229" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D229" s="17"/>
       <c r="E229"/>
       <c r="G229"/>
     </row>
-    <row r="230" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="230" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D230" s="17"/>
       <c r="E230"/>
       <c r="G230"/>
     </row>
-    <row r="231" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="231" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D231" s="17"/>
       <c r="E231"/>
       <c r="G231"/>
     </row>
-    <row r="232" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="232" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D232" s="17"/>
       <c r="E232"/>
       <c r="G232"/>
     </row>
-    <row r="233" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="233" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D233" s="17"/>
       <c r="E233"/>
       <c r="G233"/>
     </row>
-    <row r="234" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="234" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D234" s="17"/>
       <c r="E234"/>
       <c r="G234"/>
     </row>
-    <row r="235" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="235" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D235" s="17"/>
       <c r="E235"/>
       <c r="G235"/>
     </row>
-    <row r="236" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="236" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D236" s="17"/>
       <c r="E236"/>
       <c r="G236"/>
     </row>
-    <row r="237" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="237" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D237" s="17"/>
       <c r="E237"/>
       <c r="G237"/>
     </row>
-    <row r="238" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="238" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D238" s="17"/>
       <c r="E238"/>
       <c r="G238"/>
     </row>
-    <row r="239" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="239" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D239" s="17"/>
       <c r="E239"/>
       <c r="G239"/>
     </row>
-    <row r="240" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="240" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D240" s="17"/>
       <c r="E240"/>
       <c r="G240"/>
     </row>
-    <row r="241" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="241" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D241" s="17"/>
       <c r="E241"/>
       <c r="G241"/>
     </row>
-    <row r="242" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="242" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D242" s="17"/>
       <c r="E242"/>
       <c r="G242"/>
     </row>
-    <row r="243" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="243" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D243" s="17"/>
       <c r="E243"/>
       <c r="G243"/>
     </row>
-    <row r="244" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="244" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D244" s="17"/>
       <c r="E244"/>
       <c r="G244"/>
     </row>
-    <row r="245" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="245" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D245" s="17"/>
       <c r="E245"/>
       <c r="G245"/>
     </row>
-    <row r="246" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="246" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D246" s="17"/>
       <c r="E246"/>
       <c r="G246"/>
     </row>
-    <row r="247" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="247" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D247" s="17"/>
       <c r="E247"/>
       <c r="G247"/>
     </row>
-    <row r="248" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="248" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D248" s="17"/>
       <c r="E248"/>
       <c r="G248"/>
     </row>
-    <row r="249" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="249" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D249" s="17"/>
       <c r="E249"/>
       <c r="G249"/>
     </row>
-    <row r="250" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="250" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D250" s="17"/>
       <c r="E250"/>
       <c r="G250"/>
     </row>
-    <row r="251" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="251" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D251" s="17"/>
       <c r="E251"/>
       <c r="G251"/>
     </row>
-    <row r="252" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="252" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D252" s="17"/>
       <c r="E252"/>
       <c r="G252"/>
     </row>
-    <row r="253" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="253" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D253" s="17"/>
       <c r="E253"/>
       <c r="G253"/>
     </row>
-    <row r="254" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="254" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D254" s="17"/>
       <c r="E254"/>
       <c r="G254"/>
     </row>
-    <row r="255" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="255" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D255" s="17"/>
       <c r="E255"/>
       <c r="G255"/>
     </row>
-    <row r="256" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="256" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D256" s="17"/>
       <c r="E256"/>
       <c r="G256"/>
     </row>
-    <row r="257" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="257" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D257" s="17"/>
       <c r="E257"/>
       <c r="G257"/>
     </row>
-    <row r="258" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="258" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D258" s="17"/>
       <c r="E258"/>
       <c r="G258"/>
     </row>
-    <row r="259" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="259" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D259" s="17"/>
       <c r="E259"/>
       <c r="G259"/>
     </row>
-    <row r="260" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="260" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D260" s="17"/>
       <c r="E260"/>
       <c r="G260"/>
     </row>
-    <row r="261" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="261" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D261" s="17"/>
       <c r="E261"/>
       <c r="G261"/>
     </row>
-    <row r="262" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="262" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D262" s="17"/>
       <c r="E262"/>
       <c r="G262"/>
     </row>
-    <row r="263" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="263" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D263" s="17"/>
       <c r="E263"/>
       <c r="G263"/>
     </row>
-    <row r="264" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="264" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D264" s="17"/>
       <c r="E264"/>
       <c r="G264"/>
     </row>
-    <row r="265" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="265" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D265" s="17"/>
       <c r="E265"/>
       <c r="G265"/>
     </row>
-    <row r="266" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="266" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D266" s="17"/>
       <c r="E266"/>
       <c r="G266"/>
     </row>
-    <row r="267" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="267" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D267" s="17"/>
       <c r="E267"/>
       <c r="G267"/>
     </row>
-    <row r="268" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="268" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D268" s="17"/>
       <c r="E268"/>
       <c r="G268"/>
     </row>
-    <row r="269" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="269" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D269" s="17"/>
       <c r="E269"/>
       <c r="G269"/>
     </row>
-    <row r="270" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="270" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D270" s="17"/>
       <c r="E270"/>
       <c r="G270"/>
     </row>
-    <row r="271" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="271" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D271" s="17"/>
       <c r="E271"/>
       <c r="G271"/>
     </row>
-    <row r="272" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="272" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D272" s="17"/>
       <c r="E272"/>
       <c r="G272"/>
     </row>
-    <row r="273" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="273" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D273" s="17"/>
       <c r="E273"/>
       <c r="G273"/>
     </row>
-    <row r="274" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="274" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D274" s="17"/>
       <c r="E274"/>
       <c r="G274"/>
     </row>
-    <row r="275" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="275" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D275" s="17"/>
       <c r="E275"/>
       <c r="G275"/>
     </row>
-    <row r="276" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="276" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D276" s="17"/>
       <c r="E276"/>
       <c r="G276"/>
     </row>
-    <row r="277" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="277" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D277" s="17"/>
       <c r="E277"/>
       <c r="G277"/>
     </row>
-    <row r="278" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="278" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D278" s="17"/>
       <c r="E278"/>
       <c r="G278"/>
     </row>
-    <row r="279" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="279" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D279" s="17"/>
       <c r="E279"/>
       <c r="G279"/>
     </row>
-    <row r="280" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="280" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D280" s="17"/>
       <c r="E280"/>
       <c r="G280"/>
     </row>
-    <row r="281" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="281" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D281" s="17"/>
       <c r="E281"/>
       <c r="G281"/>
     </row>
-    <row r="282" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="282" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D282" s="17"/>
       <c r="E282"/>
       <c r="G282"/>
     </row>
-    <row r="283" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="283" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D283" s="17"/>
       <c r="E283"/>
       <c r="G283"/>
     </row>
-    <row r="284" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="284" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D284" s="17"/>
       <c r="E284"/>
       <c r="G284"/>
     </row>
-    <row r="285" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="285" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D285" s="17"/>
       <c r="E285"/>
       <c r="G285"/>
     </row>
-    <row r="286" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="286" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D286" s="17"/>
       <c r="E286"/>
       <c r="G286"/>
     </row>
-    <row r="287" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="287" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D287" s="17"/>
       <c r="E287"/>
       <c r="G287"/>
     </row>
-    <row r="288" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="288" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D288" s="17"/>
       <c r="E288"/>
       <c r="G288"/>
     </row>
-    <row r="289" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="289" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D289" s="17"/>
       <c r="E289"/>
       <c r="G289"/>
     </row>
-    <row r="290" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="290" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D290" s="17"/>
       <c r="E290"/>
       <c r="G290"/>
     </row>
-    <row r="291" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="291" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D291" s="17"/>
       <c r="E291"/>
       <c r="G291"/>
     </row>
-    <row r="292" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="292" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D292" s="17"/>
       <c r="E292"/>
       <c r="G292"/>
     </row>
-    <row r="293" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="293" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D293" s="17"/>
       <c r="E293"/>
       <c r="G293"/>
     </row>
-    <row r="294" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="294" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D294" s="17"/>
       <c r="E294"/>
       <c r="G294"/>
     </row>
-    <row r="295" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="295" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D295" s="17"/>
       <c r="E295"/>
       <c r="G295"/>
     </row>
-    <row r="296" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="296" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D296" s="17"/>
       <c r="E296"/>
       <c r="G296"/>
     </row>
-    <row r="297" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="297" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D297" s="17"/>
       <c r="E297"/>
       <c r="G297"/>
     </row>
-    <row r="298" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="298" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D298" s="17"/>
       <c r="E298"/>
       <c r="G298"/>
     </row>
-    <row r="299" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="299" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D299" s="17"/>
       <c r="E299"/>
       <c r="G299"/>
     </row>
-    <row r="300" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="300" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D300" s="17"/>
       <c r="E300"/>
       <c r="G300"/>
     </row>
-    <row r="301" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="301" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D301" s="17"/>
       <c r="E301"/>
       <c r="G301"/>
     </row>
-    <row r="302" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="302" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D302" s="17"/>
       <c r="E302"/>
       <c r="G302"/>
     </row>
-    <row r="303" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="303" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D303" s="17"/>
       <c r="E303"/>
       <c r="G303"/>
     </row>
-    <row r="304" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="304" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D304" s="17"/>
       <c r="E304"/>
       <c r="G304"/>
     </row>
-    <row r="305" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="305" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D305" s="17"/>
       <c r="E305"/>
       <c r="G305"/>
     </row>
-    <row r="306" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="306" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D306" s="17"/>
       <c r="E306"/>
       <c r="G306"/>
     </row>
-    <row r="307" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="307" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D307" s="17"/>
       <c r="E307"/>
       <c r="G307"/>
     </row>
-    <row r="308" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="308" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D308" s="17"/>
       <c r="E308"/>
       <c r="G308"/>
     </row>
-    <row r="309" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="309" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D309" s="17"/>
       <c r="E309"/>
       <c r="G309"/>
     </row>
-    <row r="310" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="310" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D310" s="17"/>
       <c r="E310"/>
       <c r="G310"/>
     </row>
-    <row r="311" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="311" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D311" s="17"/>
       <c r="E311"/>
       <c r="G311"/>
     </row>
-    <row r="312" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="312" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D312" s="17"/>
       <c r="E312"/>
       <c r="G312"/>
     </row>
-    <row r="313" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="313" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D313" s="17"/>
       <c r="E313"/>
       <c r="G313"/>
     </row>
-    <row r="314" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="314" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D314" s="17"/>
       <c r="E314"/>
       <c r="G314"/>
     </row>
-    <row r="315" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="315" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D315" s="17"/>
       <c r="E315"/>
       <c r="G315"/>
     </row>
-    <row r="316" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="316" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D316" s="17"/>
       <c r="E316"/>
       <c r="G316"/>
     </row>
-    <row r="317" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="317" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D317" s="17"/>
       <c r="E317"/>
       <c r="G317"/>
     </row>
-    <row r="318" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="318" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D318" s="17"/>
       <c r="E318"/>
       <c r="G318"/>
     </row>
-    <row r="319" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="319" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D319" s="17"/>
       <c r="E319"/>
       <c r="G319"/>
     </row>
-    <row r="320" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="320" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D320" s="17"/>
       <c r="E320"/>
       <c r="G320"/>
     </row>
-    <row r="321" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="321" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D321" s="17"/>
       <c r="E321"/>
       <c r="G321"/>
     </row>
-    <row r="322" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="322" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D322" s="17"/>
       <c r="E322"/>
       <c r="G322"/>
     </row>
-    <row r="323" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="323" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D323" s="17"/>
       <c r="E323"/>
       <c r="G323"/>
     </row>
-    <row r="324" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="324" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D324" s="17"/>
       <c r="E324"/>
       <c r="G324"/>
     </row>
-    <row r="325" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="325" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D325" s="17"/>
       <c r="E325"/>
       <c r="G325"/>
     </row>
-    <row r="326" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="326" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D326" s="17"/>
       <c r="E326"/>
       <c r="G326"/>
     </row>
-    <row r="327" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="327" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D327" s="17"/>
       <c r="E327"/>
       <c r="G327"/>
     </row>
-    <row r="328" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="328" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D328" s="17"/>
       <c r="E328"/>
       <c r="G328"/>
     </row>
-    <row r="329" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="329" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D329" s="17"/>
       <c r="E329"/>
       <c r="G329"/>
     </row>
-    <row r="330" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="330" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D330" s="17"/>
       <c r="E330"/>
       <c r="G330"/>
     </row>
-    <row r="331" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="331" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D331" s="17"/>
       <c r="E331"/>
       <c r="G331"/>
     </row>
-    <row r="332" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="332" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D332" s="17"/>
       <c r="E332"/>
       <c r="G332"/>
     </row>
-    <row r="333" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="333" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D333" s="17"/>
       <c r="E333"/>
       <c r="G333"/>
     </row>
-    <row r="334" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="334" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D334" s="17"/>
       <c r="E334"/>
       <c r="G334"/>
     </row>
-    <row r="335" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="335" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D335" s="17"/>
       <c r="E335"/>
       <c r="G335"/>
     </row>
-    <row r="336" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="336" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D336" s="17"/>
       <c r="E336"/>
       <c r="G336"/>
     </row>
-    <row r="337" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="337" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D337" s="17"/>
       <c r="E337"/>
       <c r="G337"/>
     </row>
-    <row r="338" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="338" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D338" s="17"/>
       <c r="E338"/>
       <c r="G338"/>
     </row>
-    <row r="339" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="339" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D339" s="17"/>
       <c r="E339"/>
       <c r="G339"/>
     </row>
-    <row r="340" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="340" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D340" s="17"/>
       <c r="E340"/>
       <c r="G340"/>
     </row>
-    <row r="341" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="341" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D341" s="17"/>
       <c r="E341"/>
       <c r="G341"/>
     </row>
-    <row r="342" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="342" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D342" s="17"/>
       <c r="E342"/>
       <c r="G342"/>
     </row>
-    <row r="343" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="343" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D343" s="17"/>
       <c r="E343"/>
       <c r="G343"/>
     </row>
-    <row r="344" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="344" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D344" s="17"/>
       <c r="E344"/>
       <c r="G344"/>
     </row>
-    <row r="345" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="345" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D345" s="17"/>
       <c r="E345"/>
       <c r="G345"/>
     </row>
-    <row r="346" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="346" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D346" s="17"/>
       <c r="E346"/>
       <c r="G346"/>
     </row>
-    <row r="347" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="347" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D347" s="17"/>
       <c r="E347"/>
       <c r="G347"/>
     </row>
-    <row r="348" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="348" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D348" s="17"/>
       <c r="E348"/>
       <c r="G348"/>
     </row>
-    <row r="349" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="349" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D349" s="17"/>
       <c r="E349"/>
       <c r="G349"/>
     </row>
-    <row r="350" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="350" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D350" s="17"/>
       <c r="E350"/>
       <c r="G350"/>
     </row>
-    <row r="351" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="351" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D351" s="17"/>
       <c r="E351"/>
       <c r="G351"/>
     </row>
-    <row r="352" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="352" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D352" s="17"/>
       <c r="E352"/>
       <c r="G352"/>
     </row>
-    <row r="353" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="353" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D353" s="17"/>
       <c r="E353"/>
       <c r="G353"/>
     </row>
-    <row r="354" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="354" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D354" s="17"/>
       <c r="E354"/>
       <c r="G354"/>
     </row>
-    <row r="355" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="355" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D355" s="17"/>
       <c r="E355"/>
       <c r="G355"/>
     </row>
-    <row r="356" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="356" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D356" s="17"/>
       <c r="E356"/>
       <c r="G356"/>
     </row>
-    <row r="357" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="357" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D357" s="17"/>
       <c r="E357"/>
       <c r="G357"/>
     </row>
-    <row r="358" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="358" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D358" s="17"/>
       <c r="E358"/>
       <c r="G358"/>
     </row>
-    <row r="359" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="359" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D359" s="17"/>
       <c r="E359"/>
       <c r="G359"/>
     </row>
-    <row r="360" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="360" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D360" s="17"/>
       <c r="E360"/>
       <c r="G360"/>
     </row>
-    <row r="361" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="361" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D361" s="17"/>
       <c r="E361"/>
       <c r="G361"/>
     </row>
-    <row r="362" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="362" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D362" s="17"/>
       <c r="E362"/>
       <c r="G362"/>
     </row>
-    <row r="363" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="363" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D363" s="17"/>
       <c r="E363"/>
       <c r="G363"/>
     </row>
-    <row r="364" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="364" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D364" s="17"/>
       <c r="E364"/>
       <c r="G364"/>
     </row>
-    <row r="365" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="365" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D365" s="17"/>
       <c r="E365"/>
       <c r="G365"/>
     </row>
-    <row r="366" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="366" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D366" s="17"/>
       <c r="E366"/>
       <c r="G366"/>
     </row>
-    <row r="367" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="367" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D367" s="17"/>
       <c r="E367"/>
       <c r="G367"/>
     </row>
-    <row r="368" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="368" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D368" s="17"/>
       <c r="E368"/>
       <c r="G368"/>
     </row>
-    <row r="369" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="369" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D369" s="17"/>
       <c r="E369"/>
       <c r="G369"/>
     </row>
-    <row r="370" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="370" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D370" s="17"/>
       <c r="E370"/>
       <c r="G370"/>
     </row>
-    <row r="371" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="371" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D371" s="17"/>
       <c r="E371"/>
       <c r="G371"/>
     </row>
-    <row r="372" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="372" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D372" s="17"/>
       <c r="E372"/>
       <c r="G372"/>
     </row>
-    <row r="373" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="373" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D373" s="17"/>
       <c r="E373"/>
       <c r="G373"/>
     </row>
-    <row r="374" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="374" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D374" s="17"/>
       <c r="E374"/>
       <c r="G374"/>
     </row>
-    <row r="375" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="375" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D375" s="17"/>
       <c r="E375"/>
       <c r="G375"/>
     </row>
-    <row r="376" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="376" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D376" s="17"/>
       <c r="E376"/>
       <c r="G376"/>
     </row>
-    <row r="377" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="377" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D377" s="17"/>
       <c r="E377"/>
       <c r="G377"/>
     </row>
-    <row r="378" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="378" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D378" s="17"/>
       <c r="E378"/>
       <c r="G378"/>
     </row>
-    <row r="379" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="379" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D379" s="17"/>
       <c r="E379"/>
       <c r="G379"/>
     </row>
-    <row r="380" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="380" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D380" s="17"/>
       <c r="E380"/>
       <c r="G380"/>
     </row>
-    <row r="381" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="381" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D381" s="17"/>
       <c r="E381"/>
       <c r="G381"/>
     </row>
-    <row r="382" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="382" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D382" s="17"/>
       <c r="E382"/>
       <c r="G382"/>
     </row>
-    <row r="383" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="383" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D383" s="17"/>
       <c r="E383"/>
       <c r="G383"/>
     </row>
-    <row r="384" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="384" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D384" s="17"/>
       <c r="E384"/>
       <c r="G384"/>
     </row>
-    <row r="385" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="385" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D385" s="17"/>
       <c r="E385"/>
       <c r="G385"/>
     </row>
-    <row r="386" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="386" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D386" s="17"/>
       <c r="E386"/>
       <c r="G386"/>
     </row>
-    <row r="387" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="387" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D387" s="17"/>
       <c r="E387"/>
       <c r="G387"/>
     </row>
-    <row r="388" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="388" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D388" s="17"/>
       <c r="E388"/>
       <c r="G388"/>
     </row>
-    <row r="389" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="389" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D389" s="17"/>
       <c r="E389"/>
       <c r="G389"/>
     </row>
-    <row r="390" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="390" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D390" s="17"/>
       <c r="E390"/>
       <c r="G390"/>
     </row>
-    <row r="391" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="391" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D391" s="17"/>
       <c r="E391"/>
       <c r="G391"/>
     </row>
-    <row r="392" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="392" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D392" s="17"/>
       <c r="E392"/>
       <c r="G392"/>
     </row>
-    <row r="393" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="393" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D393" s="17"/>
       <c r="E393"/>
       <c r="G393"/>
     </row>
-    <row r="394" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="394" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D394" s="17"/>
       <c r="E394"/>
       <c r="G394"/>
     </row>
-    <row r="395" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="395" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D395" s="17"/>
       <c r="E395"/>
       <c r="G395"/>
     </row>
-    <row r="396" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="396" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D396" s="17"/>
       <c r="E396"/>
       <c r="G396"/>
     </row>
-    <row r="397" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="397" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D397" s="17"/>
       <c r="E397"/>
       <c r="G397"/>
     </row>
-    <row r="398" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="398" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D398" s="17"/>
       <c r="E398"/>
       <c r="G398"/>
     </row>
-    <row r="399" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="399" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D399" s="17"/>
       <c r="E399"/>
       <c r="G399"/>
     </row>
-    <row r="400" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="400" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D400" s="17"/>
       <c r="E400"/>
       <c r="G400"/>
     </row>
-    <row r="401" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="401" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D401" s="17"/>
       <c r="E401"/>
       <c r="G401"/>
     </row>
-    <row r="402" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="402" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D402" s="17"/>
       <c r="E402"/>
       <c r="G402"/>
     </row>
-    <row r="403" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="403" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D403" s="17"/>
       <c r="E403"/>
       <c r="G403"/>
     </row>
-    <row r="404" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="404" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D404" s="17"/>
       <c r="E404"/>
       <c r="G404"/>
     </row>
-    <row r="405" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="405" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D405" s="17"/>
       <c r="E405"/>
       <c r="G405"/>
     </row>
-    <row r="406" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="406" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D406" s="17"/>
       <c r="E406"/>
       <c r="G406"/>
     </row>
-    <row r="407" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="407" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D407" s="17"/>
       <c r="E407"/>
       <c r="G407"/>
     </row>
-    <row r="408" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="408" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D408" s="17"/>
       <c r="E408"/>
       <c r="G408"/>
     </row>
-    <row r="409" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="409" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D409" s="17"/>
       <c r="E409"/>
       <c r="G409"/>
     </row>
-    <row r="410" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="410" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D410" s="17"/>
       <c r="E410"/>
       <c r="G410"/>
     </row>
-    <row r="411" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="411" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D411" s="17"/>
       <c r="E411"/>
       <c r="G411"/>
     </row>
-    <row r="412" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="412" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D412" s="17"/>
       <c r="E412"/>
       <c r="G412"/>
     </row>
-    <row r="413" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="413" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D413" s="17"/>
       <c r="E413"/>
       <c r="G413"/>
     </row>
-    <row r="414" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="414" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D414" s="17"/>
       <c r="E414"/>
       <c r="G414"/>
     </row>
-    <row r="415" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="415" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D415" s="17"/>
       <c r="E415"/>
       <c r="G415"/>
     </row>
-    <row r="416" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="416" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D416" s="17"/>
       <c r="E416"/>
       <c r="G416"/>
     </row>
-    <row r="417" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="417" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D417" s="17"/>
       <c r="E417"/>
       <c r="G417"/>
     </row>
-    <row r="418" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="418" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D418" s="17"/>
       <c r="E418"/>
       <c r="G418"/>
     </row>
-    <row r="419" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="419" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D419" s="17"/>
       <c r="E419"/>
       <c r="G419"/>
     </row>
-    <row r="420" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="420" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D420" s="17"/>
       <c r="E420"/>
       <c r="G420"/>
     </row>
-    <row r="421" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="421" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D421" s="17"/>
       <c r="E421"/>
       <c r="G421"/>
     </row>
-    <row r="422" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="422" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D422" s="17"/>
       <c r="E422"/>
       <c r="G422"/>
     </row>
-    <row r="423" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="423" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D423" s="17"/>
       <c r="E423"/>
       <c r="G423"/>
     </row>
-    <row r="424" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="424" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D424" s="17"/>
       <c r="E424"/>
       <c r="G424"/>
     </row>
-    <row r="425" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="425" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D425" s="17"/>
       <c r="E425"/>
       <c r="G425"/>
     </row>
-    <row r="426" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="426" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D426" s="17"/>
       <c r="E426"/>
       <c r="G426"/>
     </row>
-    <row r="427" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="427" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D427" s="17"/>
       <c r="E427"/>
       <c r="G427"/>
     </row>
-    <row r="428" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="428" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D428" s="17"/>
       <c r="E428"/>
       <c r="G428"/>
     </row>
-    <row r="429" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="429" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D429" s="17"/>
       <c r="E429"/>
       <c r="G429"/>
     </row>
-    <row r="430" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="430" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D430" s="17"/>
       <c r="E430"/>
       <c r="G430"/>
     </row>
-    <row r="431" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="431" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D431" s="17"/>
       <c r="E431"/>
       <c r="G431"/>
     </row>
-    <row r="432" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="432" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D432" s="17"/>
       <c r="E432"/>
       <c r="G432"/>
     </row>
-    <row r="433" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="433" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D433" s="17"/>
       <c r="E433"/>
       <c r="G433"/>
     </row>
-    <row r="434" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="434" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D434" s="17"/>
       <c r="E434"/>
       <c r="G434"/>
     </row>
-    <row r="435" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="435" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D435" s="17"/>
       <c r="E435"/>
       <c r="G435"/>
     </row>
-    <row r="436" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="436" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D436" s="17"/>
       <c r="E436"/>
       <c r="G436"/>
     </row>
-    <row r="437" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="437" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D437" s="17"/>
       <c r="E437"/>
       <c r="G437"/>
     </row>
-    <row r="438" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="438" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D438" s="17"/>
       <c r="E438"/>
       <c r="G438"/>
     </row>
-    <row r="439" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="439" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D439" s="17"/>
       <c r="E439"/>
       <c r="G439"/>
     </row>
-    <row r="440" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="440" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D440" s="17"/>
       <c r="E440"/>
       <c r="G440"/>
     </row>
-    <row r="441" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="441" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D441" s="17"/>
       <c r="E441"/>
       <c r="G441"/>
     </row>
-    <row r="442" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="442" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D442" s="17"/>
       <c r="E442"/>
       <c r="G442"/>
     </row>
-    <row r="443" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="443" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D443" s="17"/>
       <c r="E443"/>
       <c r="G443"/>
     </row>
-    <row r="444" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="444" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D444" s="17"/>
       <c r="E444"/>
       <c r="G444"/>
     </row>
-    <row r="445" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="445" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D445" s="17"/>
       <c r="E445"/>
       <c r="G445"/>
     </row>
-    <row r="446" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="446" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D446" s="17"/>
       <c r="E446"/>
       <c r="G446"/>
     </row>
-    <row r="447" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="447" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D447" s="17"/>
       <c r="E447"/>
       <c r="G447"/>
     </row>
-    <row r="448" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="448" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D448" s="17"/>
       <c r="E448"/>
       <c r="G448"/>
     </row>
-    <row r="449" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="449" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D449" s="17"/>
       <c r="E449"/>
       <c r="G449"/>
     </row>
-    <row r="450" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="450" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D450" s="17"/>
       <c r="E450"/>
       <c r="G450"/>
     </row>
-    <row r="451" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="451" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D451" s="17"/>
       <c r="E451"/>
       <c r="G451"/>
     </row>
-    <row r="452" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="452" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D452" s="17"/>
       <c r="E452"/>
       <c r="G452"/>
     </row>
-    <row r="453" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="453" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D453" s="17"/>
       <c r="E453"/>
       <c r="G453"/>
     </row>
-    <row r="454" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="454" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D454" s="17"/>
       <c r="E454"/>
       <c r="G454"/>
     </row>
-    <row r="455" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="455" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D455" s="17"/>
       <c r="E455"/>
       <c r="G455"/>
     </row>
-    <row r="456" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="456" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D456" s="17"/>
       <c r="E456"/>
       <c r="G456"/>
     </row>
-    <row r="457" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="457" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D457" s="17"/>
       <c r="E457"/>
       <c r="G457"/>
     </row>
-    <row r="458" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="458" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D458" s="17"/>
       <c r="E458"/>
       <c r="G458"/>
     </row>
-    <row r="459" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="459" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D459" s="17"/>
       <c r="E459"/>
       <c r="G459"/>
     </row>
-    <row r="460" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="460" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D460" s="17"/>
       <c r="E460"/>
       <c r="G460"/>
     </row>
-    <row r="461" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="461" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D461" s="17"/>
       <c r="E461"/>
       <c r="G461"/>
     </row>
-    <row r="462" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="462" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D462" s="17"/>
       <c r="E462"/>
       <c r="G462"/>
     </row>
-    <row r="463" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="463" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D463" s="17"/>
       <c r="E463"/>
       <c r="G463"/>
     </row>
-    <row r="464" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="464" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D464" s="17"/>
       <c r="E464"/>
       <c r="G464"/>
     </row>
-    <row r="465" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="465" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D465" s="17"/>
       <c r="E465"/>
       <c r="G465"/>
     </row>
-    <row r="466" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="466" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D466" s="17"/>
       <c r="E466"/>
       <c r="G466"/>
     </row>
-    <row r="467" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="467" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D467" s="17"/>
       <c r="E467"/>
       <c r="G467"/>
     </row>
-    <row r="468" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="468" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D468" s="17"/>
       <c r="E468"/>
       <c r="G468"/>
     </row>
-    <row r="469" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="469" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D469" s="17"/>
       <c r="E469"/>
       <c r="G469"/>
     </row>
-    <row r="470" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="470" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D470" s="17"/>
       <c r="E470"/>
       <c r="G470"/>
     </row>
-    <row r="471" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="471" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D471" s="17"/>
       <c r="E471"/>
       <c r="G471"/>
     </row>
-    <row r="472" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="472" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D472" s="17"/>
       <c r="E472"/>
       <c r="G472"/>
     </row>
-    <row r="473" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="473" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D473" s="17"/>
       <c r="E473"/>
       <c r="G473"/>
     </row>
-    <row r="474" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="474" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D474" s="17"/>
       <c r="E474"/>
       <c r="G474"/>
     </row>
-    <row r="475" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="475" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D475" s="17"/>
       <c r="E475"/>
       <c r="G475"/>
     </row>
-    <row r="476" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="476" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D476" s="17"/>
       <c r="E476"/>
       <c r="G476"/>
     </row>
-    <row r="477" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="477" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D477" s="17"/>
       <c r="E477"/>
       <c r="G477"/>
     </row>
-    <row r="478" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="478" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D478" s="17"/>
       <c r="E478"/>
       <c r="G478"/>
     </row>
-    <row r="479" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="479" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D479" s="17"/>
       <c r="E479"/>
       <c r="G479"/>
     </row>
-    <row r="480" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="480" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D480" s="17"/>
       <c r="E480"/>
       <c r="G480"/>
     </row>
-    <row r="481" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="481" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D481" s="17"/>
       <c r="E481"/>
       <c r="G481"/>
     </row>
-    <row r="482" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="482" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D482" s="17"/>
       <c r="E482"/>
       <c r="G482"/>
     </row>
-    <row r="483" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="483" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D483" s="17"/>
       <c r="E483"/>
       <c r="G483"/>
     </row>
-    <row r="484" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="484" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D484" s="17"/>
       <c r="E484"/>
       <c r="G484"/>
     </row>
-    <row r="485" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="485" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D485" s="17"/>
       <c r="E485"/>
       <c r="G485"/>
     </row>
-    <row r="486" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="486" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D486" s="17"/>
       <c r="E486"/>
       <c r="G486"/>
     </row>
-    <row r="487" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="487" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D487" s="17"/>
       <c r="E487"/>
       <c r="G487"/>
     </row>
-    <row r="488" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="488" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D488" s="17"/>
       <c r="E488"/>
       <c r="G488"/>
     </row>
-    <row r="489" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="489" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D489" s="17"/>
       <c r="E489"/>
       <c r="G489"/>
     </row>
-    <row r="490" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="490" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D490" s="17"/>
       <c r="E490"/>
       <c r="G490"/>
     </row>
-    <row r="491" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="491" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D491" s="17"/>
       <c r="E491"/>
       <c r="G491"/>
     </row>
-    <row r="492" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="492" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D492" s="17"/>
       <c r="E492"/>
       <c r="G492"/>
     </row>
-    <row r="493" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="493" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D493" s="17"/>
       <c r="E493"/>
       <c r="G493"/>
     </row>
-    <row r="494" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="494" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D494" s="17"/>
       <c r="E494"/>
       <c r="G494"/>
     </row>
-    <row r="495" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="495" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D495" s="17"/>
       <c r="E495"/>
       <c r="G495"/>
     </row>
-    <row r="496" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="496" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D496" s="17"/>
       <c r="E496"/>
       <c r="G496"/>
     </row>
-    <row r="497" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="497" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D497" s="17"/>
       <c r="E497"/>
       <c r="G497"/>
     </row>
-    <row r="498" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="498" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D498" s="17"/>
       <c r="E498"/>
       <c r="G498"/>
     </row>
-    <row r="499" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="499" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D499" s="17"/>
       <c r="E499"/>
       <c r="G499"/>
     </row>
-    <row r="500" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="500" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D500" s="17"/>
       <c r="E500"/>
       <c r="G500"/>
     </row>
-    <row r="501" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="501" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D501" s="17"/>
       <c r="E501"/>
       <c r="G501"/>
     </row>
-    <row r="502" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="502" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D502" s="17"/>
       <c r="E502"/>
       <c r="G502"/>
     </row>
-    <row r="503" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="503" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D503" s="17"/>
       <c r="E503"/>
       <c r="G503"/>
     </row>
-    <row r="504" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="504" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D504" s="17"/>
       <c r="E504"/>
       <c r="G504"/>
     </row>
-    <row r="505" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="505" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D505" s="17"/>
       <c r="E505"/>
       <c r="G505"/>
     </row>
-    <row r="506" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="506" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D506" s="17"/>
       <c r="E506"/>
       <c r="G506"/>
     </row>
-    <row r="507" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="507" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D507" s="17"/>
       <c r="E507"/>
       <c r="G507"/>
     </row>
-    <row r="508" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="508" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D508" s="17"/>
       <c r="E508"/>
       <c r="G508"/>
     </row>
-    <row r="509" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="509" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D509" s="17"/>
       <c r="E509"/>
       <c r="G509"/>
     </row>
-    <row r="510" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="510" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D510" s="17"/>
       <c r="E510"/>
       <c r="G510"/>
     </row>
-    <row r="511" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="511" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D511" s="17"/>
       <c r="E511"/>
       <c r="G511"/>
     </row>
-    <row r="512" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="512" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D512" s="17"/>
       <c r="E512"/>
       <c r="G512"/>
     </row>
-    <row r="513" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="513" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D513" s="17"/>
       <c r="E513"/>
       <c r="G513"/>
     </row>
-    <row r="514" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="514" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D514" s="17"/>
       <c r="E514"/>
       <c r="G514"/>
     </row>
-    <row r="515" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="515" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D515" s="17"/>
       <c r="E515"/>
       <c r="G515"/>
     </row>
-    <row r="516" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="516" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D516" s="17"/>
       <c r="E516"/>
       <c r="G516"/>
     </row>
-    <row r="517" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="517" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D517" s="17"/>
       <c r="E517"/>
       <c r="G517"/>
     </row>
-    <row r="518" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="518" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D518" s="17"/>
       <c r="E518"/>
       <c r="G518"/>
     </row>
-    <row r="519" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="519" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D519" s="17"/>
       <c r="E519"/>
       <c r="G519"/>
     </row>
-    <row r="520" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="520" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D520" s="17"/>
       <c r="E520"/>
       <c r="G520"/>
     </row>
-    <row r="521" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="521" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D521" s="17"/>
       <c r="E521"/>
       <c r="G521"/>
     </row>
-    <row r="522" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="522" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D522" s="17"/>
       <c r="E522"/>
       <c r="G522"/>
     </row>
-    <row r="523" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="523" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D523" s="17"/>
       <c r="E523"/>
       <c r="G523"/>
     </row>
-    <row r="524" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="524" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D524" s="17"/>
       <c r="E524"/>
       <c r="G524"/>
     </row>
-    <row r="525" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="525" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D525" s="17"/>
       <c r="E525"/>
       <c r="G525"/>
     </row>
-    <row r="526" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="526" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D526" s="17"/>
       <c r="E526"/>
       <c r="G526"/>
     </row>
-    <row r="527" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="527" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D527" s="17"/>
       <c r="E527"/>
       <c r="G527"/>
     </row>
-    <row r="528" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="528" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D528" s="17"/>
       <c r="E528"/>
       <c r="G528"/>
     </row>
-    <row r="529" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="529" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D529" s="17"/>
       <c r="E529"/>
       <c r="G529"/>
     </row>
-    <row r="530" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="530" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D530" s="17"/>
       <c r="E530"/>
       <c r="G530"/>
     </row>
-    <row r="531" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="531" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D531" s="17"/>
       <c r="E531"/>
       <c r="G531"/>
     </row>
-    <row r="532" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="532" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D532" s="17"/>
       <c r="E532"/>
       <c r="G532"/>
     </row>
-    <row r="533" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="533" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D533" s="17"/>
       <c r="E533"/>
       <c r="G533"/>
     </row>
-    <row r="534" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="534" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D534" s="17"/>
       <c r="E534"/>
       <c r="G534"/>
     </row>
-    <row r="535" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="535" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D535" s="17"/>
       <c r="E535"/>
       <c r="G535"/>
     </row>
-    <row r="536" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="536" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D536" s="17"/>
       <c r="E536"/>
       <c r="G536"/>
     </row>
-    <row r="537" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="537" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D537" s="17"/>
       <c r="E537"/>
       <c r="G537"/>
     </row>
-    <row r="538" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="538" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D538" s="17"/>
       <c r="E538"/>
       <c r="G538"/>
     </row>
-    <row r="539" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="539" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D539" s="17"/>
       <c r="E539"/>
       <c r="G539"/>
     </row>
-    <row r="540" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="540" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D540" s="17"/>
       <c r="E540"/>
       <c r="G540"/>
     </row>
-    <row r="541" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="541" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D541" s="17"/>
       <c r="E541"/>
       <c r="G541"/>
     </row>
-    <row r="542" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="542" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D542" s="17"/>
       <c r="E542"/>
       <c r="G542"/>
     </row>
-    <row r="543" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="543" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D543" s="17"/>
       <c r="E543"/>
       <c r="G543"/>
     </row>
-    <row r="544" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="544" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D544" s="17"/>
       <c r="E544"/>
       <c r="G544"/>
     </row>
-    <row r="545" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="545" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D545" s="17"/>
       <c r="E545"/>
       <c r="G545"/>
     </row>
-    <row r="546" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="546" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D546" s="17"/>
       <c r="E546"/>
       <c r="G546"/>
     </row>
-    <row r="547" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="547" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D547" s="17"/>
       <c r="E547"/>
       <c r="G547"/>
     </row>
-    <row r="548" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="548" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D548" s="17"/>
       <c r="E548"/>
       <c r="G548"/>
     </row>
-    <row r="549" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="549" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D549" s="17"/>
       <c r="E549"/>
       <c r="G549"/>
     </row>
-    <row r="550" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="550" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D550" s="17"/>
       <c r="E550"/>
       <c r="G550"/>
     </row>
-    <row r="551" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="551" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D551" s="17"/>
       <c r="E551"/>
       <c r="G551"/>
     </row>
-    <row r="552" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="552" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D552" s="17"/>
       <c r="E552"/>
       <c r="G552"/>
     </row>
-    <row r="553" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="553" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D553" s="17"/>
       <c r="E553"/>
       <c r="G553"/>
     </row>
-    <row r="554" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="554" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D554" s="17"/>
       <c r="E554"/>
       <c r="G554"/>
     </row>
-    <row r="555" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="555" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D555" s="17"/>
       <c r="E555"/>
       <c r="G555"/>
     </row>
-    <row r="556" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="556" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D556" s="17"/>
       <c r="E556"/>
       <c r="G556"/>
     </row>
-    <row r="557" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="557" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D557" s="17"/>
       <c r="E557"/>
       <c r="G557"/>
     </row>
-    <row r="558" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="558" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D558" s="17"/>
       <c r="E558"/>
       <c r="G558"/>
     </row>
-    <row r="559" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="559" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D559" s="17"/>
       <c r="E559"/>
       <c r="G559"/>
     </row>
-    <row r="560" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="560" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D560" s="17"/>
       <c r="E560"/>
       <c r="G560"/>
     </row>
-    <row r="561" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="561" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D561" s="17"/>
       <c r="E561"/>
       <c r="G561"/>
     </row>
-    <row r="562" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="562" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D562" s="17"/>
       <c r="E562"/>
       <c r="G562"/>
     </row>
-    <row r="563" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="563" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D563" s="17"/>
       <c r="E563"/>
       <c r="G563"/>
     </row>
-    <row r="564" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="564" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D564" s="17"/>
       <c r="E564"/>
       <c r="G564"/>
     </row>
-    <row r="565" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="565" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D565" s="17"/>
       <c r="E565"/>
       <c r="G565"/>
     </row>
-    <row r="566" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="566" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D566" s="17"/>
       <c r="E566"/>
       <c r="G566"/>
     </row>
-    <row r="567" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="567" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D567" s="17"/>
       <c r="E567"/>
       <c r="G567"/>
     </row>
-    <row r="568" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="568" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D568" s="17"/>
       <c r="E568"/>
       <c r="G568"/>
     </row>
-    <row r="569" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="569" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D569" s="17"/>
       <c r="E569"/>
       <c r="G569"/>
     </row>
-    <row r="570" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="570" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D570" s="17"/>
       <c r="E570"/>
       <c r="G570"/>
     </row>
-    <row r="571" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="571" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D571" s="17"/>
       <c r="E571"/>
       <c r="G571"/>
     </row>
-    <row r="572" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="572" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D572" s="17"/>
       <c r="E572"/>
       <c r="G572"/>
     </row>
-    <row r="573" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="573" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D573" s="17"/>
       <c r="E573"/>
       <c r="G573"/>
     </row>
-    <row r="574" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="574" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D574" s="17"/>
       <c r="E574"/>
       <c r="G574"/>
     </row>
-    <row r="575" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="575" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D575" s="17"/>
       <c r="E575"/>
       <c r="G575"/>
     </row>
-    <row r="576" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="576" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D576" s="17"/>
       <c r="E576"/>
       <c r="G576"/>
     </row>
-    <row r="577" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="577" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D577" s="17"/>
       <c r="E577"/>
       <c r="G577"/>
     </row>
-    <row r="578" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="578" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D578" s="17"/>
       <c r="E578"/>
       <c r="G578"/>
     </row>
-    <row r="579" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="579" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D579" s="17"/>
       <c r="E579"/>
       <c r="G579"/>
     </row>
-    <row r="580" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="580" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D580" s="17"/>
       <c r="E580"/>
       <c r="G580"/>
     </row>
-    <row r="581" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="581" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D581" s="17"/>
       <c r="E581"/>
       <c r="G581"/>
     </row>
-    <row r="582" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="582" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D582" s="17"/>
       <c r="E582"/>
       <c r="G582"/>
     </row>
-    <row r="583" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="583" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D583" s="17"/>
       <c r="E583"/>
       <c r="G583"/>
     </row>
-    <row r="584" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="584" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D584" s="17"/>
       <c r="E584"/>
       <c r="G584"/>
     </row>
-    <row r="585" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="585" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D585" s="17"/>
       <c r="E585"/>
       <c r="G585"/>
     </row>
-    <row r="586" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="586" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D586" s="17"/>
       <c r="E586"/>
       <c r="G586"/>
     </row>
-    <row r="587" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="587" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D587" s="17"/>
       <c r="E587"/>
       <c r="G587"/>
     </row>
-    <row r="588" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="588" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D588" s="17"/>
       <c r="E588"/>
       <c r="G588"/>
     </row>
-    <row r="589" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="589" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D589" s="17"/>
       <c r="E589"/>
       <c r="G589"/>
     </row>
-    <row r="590" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="590" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D590" s="17"/>
       <c r="E590"/>
       <c r="G590"/>
     </row>
-    <row r="591" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="591" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D591" s="17"/>
       <c r="E591"/>
       <c r="G591"/>
     </row>
-    <row r="592" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="592" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D592" s="17"/>
       <c r="E592"/>
       <c r="G592"/>
     </row>
-    <row r="593" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="593" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D593" s="17"/>
       <c r="E593"/>
       <c r="G593"/>
     </row>
-    <row r="594" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="594" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D594" s="17"/>
       <c r="E594"/>
       <c r="G594"/>
     </row>
-    <row r="595" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="595" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D595" s="17"/>
       <c r="E595"/>
       <c r="G595"/>
     </row>
-    <row r="596" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="596" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D596" s="17"/>
       <c r="E596"/>
       <c r="G596"/>
     </row>
-    <row r="597" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="597" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D597" s="17"/>
       <c r="E597"/>
       <c r="G597"/>
     </row>
-    <row r="598" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="598" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D598" s="17"/>
       <c r="E598"/>
       <c r="G598"/>
     </row>
-    <row r="599" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="599" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D599" s="17"/>
       <c r="E599"/>
       <c r="G599"/>
     </row>
-    <row r="600" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="600" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D600" s="17"/>
       <c r="E600"/>
       <c r="G600"/>
     </row>
-    <row r="601" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="601" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D601" s="17"/>
       <c r="E601"/>
       <c r="G601"/>
     </row>
-    <row r="602" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="602" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D602" s="17"/>
       <c r="E602"/>
       <c r="G602"/>
     </row>
-    <row r="603" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="603" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D603" s="17"/>
       <c r="E603"/>
       <c r="G603"/>
     </row>
-    <row r="604" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="604" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D604" s="17"/>
       <c r="E604"/>
       <c r="G604"/>
     </row>
-    <row r="605" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="605" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D605" s="17"/>
       <c r="E605"/>
       <c r="G605"/>
     </row>
-    <row r="606" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="606" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D606" s="17"/>
       <c r="E606"/>
       <c r="G606"/>
     </row>
-    <row r="607" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="607" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D607" s="17"/>
       <c r="E607"/>
       <c r="G607"/>
     </row>
-    <row r="608" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="608" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D608" s="17"/>
       <c r="E608"/>
       <c r="G608"/>
     </row>
-    <row r="609" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="609" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D609" s="17"/>
       <c r="E609"/>
       <c r="G609"/>
     </row>
-    <row r="610" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="610" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D610" s="17"/>
       <c r="E610"/>
       <c r="G610"/>
     </row>
-    <row r="611" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="611" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D611" s="17"/>
       <c r="E611"/>
       <c r="G611"/>
     </row>
-    <row r="612" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="612" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D612" s="17"/>
       <c r="E612"/>
       <c r="G612"/>
     </row>
-    <row r="613" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="613" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D613" s="17"/>
       <c r="E613"/>
       <c r="G613"/>
     </row>
-    <row r="614" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="614" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D614" s="17"/>
       <c r="E614"/>
       <c r="G614"/>
     </row>
-    <row r="615" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="615" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D615" s="17"/>
       <c r="E615"/>
       <c r="G615"/>
     </row>
-    <row r="616" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="616" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D616" s="17"/>
       <c r="E616"/>
       <c r="G616"/>
     </row>
-    <row r="617" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="617" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D617" s="17"/>
       <c r="E617"/>
       <c r="G617"/>
     </row>
-    <row r="618" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="618" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D618" s="17"/>
       <c r="E618"/>
       <c r="G618"/>
     </row>
-    <row r="619" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="619" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D619" s="17"/>
       <c r="E619"/>
       <c r="G619"/>
     </row>
-    <row r="620" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="620" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D620" s="17"/>
       <c r="E620"/>
       <c r="G620"/>
     </row>
-    <row r="621" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="621" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D621" s="17"/>
       <c r="E621"/>
       <c r="G621"/>
     </row>
-    <row r="622" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="622" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D622" s="17"/>
       <c r="E622"/>
       <c r="G622"/>
     </row>
-    <row r="623" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="623" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D623" s="17"/>
       <c r="E623"/>
       <c r="G623"/>
     </row>
-    <row r="624" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="624" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D624" s="17"/>
       <c r="E624"/>
       <c r="G624"/>
     </row>
-    <row r="625" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="625" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D625" s="17"/>
       <c r="E625"/>
       <c r="G625"/>
     </row>
-    <row r="626" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="626" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D626" s="17"/>
       <c r="E626"/>
       <c r="G626"/>
     </row>
-    <row r="627" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="627" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D627" s="17"/>
       <c r="E627"/>
       <c r="G627"/>
     </row>
-    <row r="628" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="628" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D628" s="17"/>
       <c r="E628"/>
       <c r="G628"/>
     </row>
-    <row r="629" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="629" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D629" s="17"/>
       <c r="E629"/>
       <c r="G629"/>
     </row>
-    <row r="630" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="630" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D630" s="17"/>
       <c r="E630"/>
       <c r="G630"/>
     </row>
-    <row r="631" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="631" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D631" s="17"/>
       <c r="E631"/>
       <c r="G631"/>
     </row>
-    <row r="632" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="632" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D632" s="17"/>
       <c r="E632"/>
       <c r="G632"/>
     </row>
-    <row r="633" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="633" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D633" s="17"/>
       <c r="E633"/>
       <c r="G633"/>
     </row>
-    <row r="634" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="634" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D634" s="17"/>
       <c r="E634"/>
       <c r="G634"/>
     </row>
-    <row r="635" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="635" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D635" s="17"/>
       <c r="E635"/>
       <c r="G635"/>
     </row>
-    <row r="636" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="636" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D636" s="17"/>
       <c r="E636"/>
       <c r="G636"/>
     </row>
-    <row r="637" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="637" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D637" s="17"/>
       <c r="E637"/>
       <c r="G637"/>
     </row>
-    <row r="638" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="638" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D638" s="17"/>
       <c r="E638"/>
       <c r="G638"/>
     </row>
-    <row r="639" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="639" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D639" s="17"/>
       <c r="E639"/>
       <c r="G639"/>
     </row>
-    <row r="640" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="640" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D640" s="17"/>
       <c r="E640"/>
       <c r="G640"/>
     </row>
-    <row r="641" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="641" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D641" s="17"/>
       <c r="E641"/>
       <c r="G641"/>
     </row>
-    <row r="642" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="642" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D642" s="17"/>
       <c r="E642"/>
       <c r="G642"/>
     </row>
-    <row r="643" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="643" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D643" s="17"/>
       <c r="E643"/>
       <c r="G643"/>
     </row>
-    <row r="644" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="644" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D644" s="17"/>
       <c r="E644"/>
       <c r="G644"/>
     </row>
-    <row r="645" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="645" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D645" s="17"/>
       <c r="E645"/>
       <c r="G645"/>
     </row>
-    <row r="646" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="646" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D646" s="17"/>
       <c r="E646"/>
       <c r="G646"/>
     </row>
-    <row r="647" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="647" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D647" s="17"/>
       <c r="E647"/>
       <c r="G647"/>
     </row>
-    <row r="648" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="648" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D648" s="17"/>
       <c r="E648"/>
       <c r="G648"/>
     </row>
-    <row r="649" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="649" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D649" s="17"/>
       <c r="E649"/>
       <c r="G649"/>
     </row>
-    <row r="650" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="650" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D650" s="17"/>
       <c r="E650"/>
       <c r="G650"/>
     </row>
-    <row r="651" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="651" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D651" s="17"/>
       <c r="E651"/>
       <c r="G651"/>
     </row>
-    <row r="652" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="652" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D652" s="17"/>
       <c r="E652"/>
       <c r="G652"/>
     </row>
-    <row r="653" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="653" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D653" s="17"/>
       <c r="E653"/>
       <c r="G653"/>
     </row>
-    <row r="654" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="654" spans="4:7" x14ac:dyDescent="0.3">
       <c r="E654"/>
       <c r="G654"/>
     </row>
-    <row r="655" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="655" spans="4:7" x14ac:dyDescent="0.3">
       <c r="E655"/>
       <c r="G655"/>
     </row>
-    <row r="656" spans="5:7" x14ac:dyDescent="0.3">
+    <row r="656" spans="4:7" x14ac:dyDescent="0.3">
       <c r="E656"/>
       <c r="G656"/>
     </row>

</xml_diff>